<commit_message>
Discovered critical error and changed pinout
</commit_message>
<xml_diff>
--- a/Electrical/driver_board/driver_board_v2/Pin_Layout_STM32_Robot_PCB.xlsx
+++ b/Electrical/driver_board/driver_board_v2/Pin_Layout_STM32_Robot_PCB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emanu\Desktop\Open-robot-arm\Electrical\driver_board\driver_board_v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85A56E7E-A9E5-4ACA-BF8F-E562D42D18E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFAD272F-66C9-4DA8-9419-CF3B027A1A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -97,9 +97,6 @@
     <t>SW = Serial Wire</t>
   </si>
   <si>
-    <t>PA13</t>
-  </si>
-  <si>
     <t>SWDIO</t>
   </si>
   <si>
@@ -179,6 +176,9 @@
   </si>
   <si>
     <t>PB8</t>
+  </si>
+  <si>
+    <t>PB15</t>
   </si>
   <si>
     <t>PA7</t>
@@ -726,16 +726,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>19</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -746,80 +746,80 @@
         <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="F10" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="F11" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="F12" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>41</v>
-      </c>
       <c r="F13" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="F14" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -833,7 +833,7 @@
         <v>55</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -847,7 +847,7 @@
         <v>57</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.25">
@@ -861,7 +861,7 @@
         <v>59</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.25">
@@ -933,7 +933,7 @@
     </row>
     <row r="24" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>25</v>
+        <v>52</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>19</v>
@@ -988,7 +988,7 @@
     </row>
     <row r="29" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>19</v>
@@ -1010,7 +1010,7 @@
     </row>
     <row r="31" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>19</v>
@@ -1054,7 +1054,7 @@
     </row>
     <row r="35" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>19</v>

</xml_diff>